<commit_message>
Update curriculum content and question banks
</commit_message>
<xml_diff>
--- a/content/Question Bank/MCQ/Unit 10 - Modules and Packages/Unit 10 - Modules and Packages - MCQ.xlsx
+++ b/content/Question Bank/MCQ/Unit 10 - Modules and Packages/Unit 10 - Modules and Packages - MCQ.xlsx
@@ -1243,7 +1243,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>A dozen loose modules in one flat folder recreates the original 'one giant file' clutter problem one level up; grouping related modules into packages lets folders mirror the natural categories of the project and gives `__init__`.py a place to curate what is meant to be used from outside.</t>
+          <t>A dozen loose modules in one flat folder recreates the original 'one giant file' clutter problem one level up; grouping related modules into packages lets folders mirror the natural categories of the project and gives `__init__.py` a place to curate what is meant to be used from outside.</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -1316,7 +1316,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>`billing.py` contains a `print(split_cost(1000, 5))` statement directly at the top level, outside any function. What happens every time another script writes import billing?</t>
+          <t>`billing.py` contains a `print(split_cost(1000, 5))` statement directly at the top level, outside any function. What happens every time another script writes `import billing`?</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>A folder containing an `__init__`.py file</t>
+          <t>A folder containing an `__init__.py` file</t>
         </is>
       </c>
       <c r="Q2" t="n">
@@ -2933,12 +2933,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>A team is setting up a new package called `tools` for their inventory system and wants the folder to be recognized as an importable package. What is the minimum required content of `__init__`.py for a folder to function as a package?</t>
+          <t>A team is setting up a new package called `tools` for their inventory system and wants the folder to be recognized as an importable package. What is the minimum required content of `__init__.py` for a folder to function as a package?</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>`__init__`.py can be completely empty; its mere presence in the folder is sufficient to mark it as a package, with no required content inside it.</t>
+          <t>`__init__.py` can be completely empty; its mere presence in the folder is sufficient to mark it as a package, with no required content inside it.</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -3011,13 +3011,13 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>In an e-commerce project's `tools` package, the file structure includes `tools/__init__`.py containing: from .billing import `split_cost`
+          <t>In an e-commerce project's `tools` package, the file structure includes `tools/__init__.py` containing: `from .billing import split_cost`
 What does this allow `main.py` to do?</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>This re-export lets `main.py` write from tools import `split_cost` directly, without separately naming the billing module, since `__init__`.py code runs when the package itself is first imported and can expose inner names at the package level.</t>
+          <t>This re-export lets `main.py` write `from tools import split_cost` directly, without separately naming the billing module, since `__init__.py` code runs when the package itself is first imported and can expose inner names at the package level.</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -3070,12 +3070,12 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Nothing changes at all; `__init__`.py code technically never actually runs</t>
+          <t>Nothing changes at all; `__init__.py` code technically never actually runs</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>`main.py` can now write from tools import `split_cost` directly, skipping the billing name</t>
+          <t>`main.py` can now write `from tools import split_cost` directly, skipping the billing name</t>
         </is>
       </c>
       <c r="Q10" t="n">
@@ -3095,7 +3095,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>A package is a folder containing related module files, plus a special file named `__init__`.py inside it; the mere presence of `__init__`.py is what tells Python to treat the folder as an importable package rather than an ordinary one.</t>
+          <t>A package is a folder containing related module files, plus a special file named `__init__.py` inside it; the mere presence of `__init__.py` is what tells Python to treat the folder as an importable package rather than an ordinary one.</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -3138,7 +3138,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>A folder of related modules plus an `__init__`.py file inside it</t>
+          <t>A folder of related modules plus an `__init__.py` file inside it</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -3581,7 +3581,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Inside an online bookstore project's `tools/__init__`.py file, a developer sees a relative import: from .billing import `split_cost`. What does the leading dot in from .billing import `split_cost` mean?</t>
+          <t>Inside an online bookstore project's `tools/__init__.py` file, a developer sees a relative import: `from .billing import split_cost`. What does the leading dot in `from .billing import split_cost` mean?</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">

</xml_diff>